<commit_message>
Daily auto backup 2026-08-24 17:10
</commit_message>
<xml_diff>
--- a/team_roster.xlsx
+++ b/team_roster.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LOP2COB\Desktop\TOTAL TIME\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FA67CC8-C52B-4A6A-B8C7-E433D167985D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E3E0B89-BB94-4F51-9D0C-0546D6C3AF5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" firstSheet="9" activeTab="9" xr2:uid="{970AEED6-FC54-4933-903B-12947F7B1334}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="9" activeTab="9" xr2:uid="{970AEED6-FC54-4933-903B-12947F7B1334}"/>
   </bookViews>
   <sheets>
     <sheet name="EHN1 D" sheetId="3" state="hidden" r:id="rId1"/>
@@ -39,10 +39,9 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId14"/>
-    <pivotCache cacheId="1" r:id="rId15"/>
+    <pivotCache cacheId="2" r:id="rId14"/>
+    <pivotCache cacheId="3" r:id="rId15"/>
   </pivotCaches>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -66,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2861" uniqueCount="594">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2861" uniqueCount="598">
   <si>
     <t>NTID</t>
   </si>
@@ -1848,6 +1847,18 @@
   </si>
   <si>
     <t>Susan Philip Deenu</t>
+  </si>
+  <si>
+    <t>Anitha Anju</t>
+  </si>
+  <si>
+    <t>Angadi Darshan Amaresh</t>
+  </si>
+  <si>
+    <t>Majhi Shouvik</t>
+  </si>
+  <si>
+    <t>Jadhav Amol</t>
   </si>
 </sst>
 </file>
@@ -8119,7 +8130,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0098736E-B170-480A-8646-B4038DDF88E3}" name="PivotTable12" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0098736E-B170-480A-8646-B4038DDF88E3}" name="PivotTable12" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B13" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="21">
     <pivotField showAll="0"/>
@@ -8229,7 +8240,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E7876BB2-FAA5-4E33-A0C3-DBF06492F213}" name="PivotTable13" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E7876BB2-FAA5-4E33-A0C3-DBF06492F213}" name="PivotTable13" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="21">
     <pivotField showAll="0"/>
@@ -8342,7 +8353,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2D21F152-1BD0-445B-A649-FB9E922322CE}" name="PivotTable14" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2D21F152-1BD0-445B-A649-FB9E922322CE}" name="PivotTable14" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:D11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="21">
     <pivotField showAll="0"/>
@@ -11182,7 +11193,7 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" s="17" t="s">
-        <v>150</v>
+        <v>596</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
@@ -11342,7 +11353,7 @@
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" s="17" t="s">
-        <v>224</v>
+        <v>594</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
@@ -11357,7 +11368,7 @@
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" s="17" t="s">
-        <v>230</v>
+        <v>595</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
@@ -11522,7 +11533,7 @@
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" s="17" t="s">
-        <v>142</v>
+        <v>597</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.35">
@@ -23472,6 +23483,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B2DE2FA78769124F84FDD7E0EC4CE68A" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="09dcf48ca891666ab2c00af7f4bf2e97">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="56a4d888-44a4-4354-b193-9d5742ce170a" xmlns:ns4="9c3a2386-fa12-446f-89ed-7b5749bf6418" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="788abaac814fef6acb3e842a1597d93d" ns3:_="" ns4:_="">
     <xsd:import namespace="56a4d888-44a4-4354-b193-9d5742ce170a"/>
@@ -23698,15 +23718,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD5DE914-35A0-4481-A533-7E8F61A0C1E8}">
   <ds:schemaRefs>
@@ -23718,6 +23729,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACF9A59E-7B3C-49C6-84F1-9A7495063C29}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F4FA2B82-9097-4ACC-A2FF-1D0AD0905FD8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -23734,12 +23753,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACF9A59E-7B3C-49C6-84F1-9A7495063C29}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>